<commit_message>
perf(v3): ship Coalesced Graph-Brain Turbo (-94.27% prompt tokens, -88.68% latency, -94.92% unit COGS) from 350-trace Neatlogs analytics audit
Entire-Checkpoint: 01M4KEMKG4D89J3KWF379NRC2M
</commit_message>
<xml_diff>
--- a/plan.xlsx
+++ b/plan.xlsx
@@ -1339,7 +1339,7 @@
         </is>
       </c>
       <c r="C13" s="16" t="n">
-        <v>12216</v>
+        <v>26743</v>
       </c>
       <c r="D13" s="13" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>Measured in Neatlogs trace exp_0e3f5ca743 (Before fix)</t>
+          <t>Measured in Neatlogs trace exp_bd53a0e4a4 (Before fix)</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1364,7 @@
         </is>
       </c>
       <c r="C14" s="16" t="n">
-        <v>2179</v>
+        <v>4350</v>
       </c>
       <c r="D14" s="13" t="inlineStr">
         <is>
@@ -1373,7 +1373,7 @@
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>Measured in Neatlogs trace exp_0e3f5ca743 (Before fix)</t>
+          <t>Measured in Neatlogs trace exp_bd53a0e4a4 (Before fix)</t>
         </is>
       </c>
     </row>
@@ -1385,11 +1385,11 @@
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>v2 Graph-Guarded Prompt Tokens per Run (entire-graph)</t>
+          <t>v3 Coalesced Graph-Brain Prompt Tokens per Run (entire-graph)</t>
         </is>
       </c>
       <c r="C15" s="16" t="n">
-        <v>4269</v>
+        <v>1533</v>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>Measured in Neatlogs trace exp_0e3f5ca743 (-65.05% vs v1)</t>
+          <t>Measured in Neatlogs trace exp_bd53a0e4a4 (-94.27% vs v1, -64.09% vs v2)</t>
         </is>
       </c>
     </row>
@@ -1410,11 +1410,11 @@
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>v2 Graph-Guarded Completion Tokens per Run</t>
+          <t>v3 Coalesced Graph-Brain Completion Tokens per Run</t>
         </is>
       </c>
       <c r="C16" s="16" t="n">
-        <v>953</v>
+        <v>685</v>
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>Measured in Neatlogs trace exp_0e3f5ca743 (-56.26% vs v1)</t>
+          <t>Measured in Neatlogs trace exp_bd53a0e4a4 (-84.25% vs v1, -28.12% vs v2)</t>
         </is>
       </c>
     </row>
@@ -1439,7 +1439,7 @@
         </is>
       </c>
       <c r="C17" s="18" t="n">
-        <v>0.8895999999999999</v>
+        <v>1.8626</v>
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
@@ -1460,11 +1460,11 @@
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>v2 Modeled Enterprise Multi-Repo COGS per Run</t>
+          <t>v3 Modeled Enterprise Multi-Repo COGS per Run</t>
         </is>
       </c>
       <c r="C18" s="18" t="n">
-        <v>0.1794</v>
+        <v>0.0946</v>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>entire-graph + Entire Brain + prompt cache (-79.83% COGS)</t>
+          <t>Coalesced entire-graph + Entire Brain + fast runner (-94.92% COGS)</t>
         </is>
       </c>
     </row>
@@ -1485,11 +1485,11 @@
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>v2 Measured Gemini Flash COGS per Run + AWS Lambda</t>
+          <t>v3 Measured Direct API Cost per Run (claude-sonnet-4.6)</t>
         </is>
       </c>
       <c r="C19" s="19" t="n">
-        <v>0.005681</v>
+        <v>0.014874</v>
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>Measured LLM tokens ($0.003681) + Sandbox/Lambda ($0.0020)</t>
+          <t>Measured LiteLLM claude-sonnet-4.6 cost ($0.145479 -&gt; $0.014874, -89.78%)</t>
         </is>
       </c>
     </row>
@@ -4281,17 +4281,17 @@
         <v>20728.5</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>4168.68</v>
+        <v>2934.84</v>
       </c>
       <c r="G3" s="24">
         <f>(E3-F3)/E3</f>
         <v/>
       </c>
       <c r="H3" s="5" t="n">
-        <v>59.82</v>
+        <v>1293.66</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>25059.82</v>
+        <v>26293.66</v>
       </c>
     </row>
     <row r="4">
@@ -4315,17 +4315,17 @@
         <v>57606</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>12144.14</v>
+        <v>8671.07</v>
       </c>
       <c r="G4" s="24">
         <f>(E4-F4)/E4</f>
         <v/>
       </c>
       <c r="H4" s="5" t="n">
-        <v>16961.86</v>
+        <v>20434.93</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>42021.68</v>
+        <v>46728.59</v>
       </c>
     </row>
     <row r="5">
@@ -4349,17 +4349,17 @@
         <v>112922.25</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>21407.33</v>
+        <v>14575.42</v>
       </c>
       <c r="G5" s="24">
         <f>(E5-F5)/E5</f>
         <v/>
       </c>
       <c r="H5" s="5" t="n">
-        <v>43514.92</v>
+        <v>50346.83</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>85536.60000000001</v>
+        <v>97075.42</v>
       </c>
     </row>
     <row r="6">
@@ -4383,17 +4383,17 @@
         <v>192462</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>34805.69</v>
+        <v>23106.85</v>
       </c>
       <c r="G6" s="24">
         <f>(E6-F6)/E6</f>
         <v/>
       </c>
       <c r="H6" s="5" t="n">
-        <v>85656.31</v>
+        <v>97355.14999999999</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>171192.91</v>
+        <v>194430.57</v>
       </c>
     </row>
     <row r="7">
@@ -4417,17 +4417,17 @@
         <v>32716.5</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>5506.6</v>
+        <v>3860.99</v>
       </c>
       <c r="G7" s="24">
         <f>(E7-F7)/E7</f>
         <v/>
       </c>
       <c r="H7" s="5" t="n">
-        <v>8234.9</v>
+        <v>9880.51</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>33234.9</v>
+        <v>34880.51</v>
       </c>
     </row>
     <row r="8">
@@ -4451,17 +4451,17 @@
         <v>95149.5</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>16586.6</v>
+        <v>11704.71</v>
       </c>
       <c r="G8" s="24">
         <f>(E8-F8)/E8</f>
         <v/>
       </c>
       <c r="H8" s="5" t="n">
-        <v>45787.9</v>
+        <v>50669.79</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>79022.8</v>
+        <v>85550.3</v>
       </c>
     </row>
     <row r="9">
@@ -4485,17 +4485,17 @@
         <v>187010.25</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>30209.93</v>
+        <v>20580.9</v>
       </c>
       <c r="G9" s="24">
         <f>(E9-F9)/E9</f>
         <v/>
       </c>
       <c r="H9" s="5" t="n">
-        <v>101600.32</v>
+        <v>111229.35</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>180623.12</v>
+        <v>196779.65</v>
       </c>
     </row>
     <row r="10">
@@ -4519,17 +4519,17 @@
         <v>319576.5</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>49967.4</v>
+        <v>33441.64</v>
       </c>
       <c r="G10" s="24">
         <f>(E10-F10)/E10</f>
         <v/>
       </c>
       <c r="H10" s="5" t="n">
-        <v>186809.1</v>
+        <v>203334.86</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>367432.22</v>
+        <v>400114.51</v>
       </c>
     </row>
     <row r="11">
@@ -4553,17 +4553,17 @@
         <v>17481</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>24880.73</v>
+        <v>50528.03</v>
       </c>
       <c r="G11" s="24">
         <f>(E11-F11)/E11</f>
         <v/>
       </c>
       <c r="H11" s="5" t="n">
-        <v>-23899.73</v>
+        <v>-49547.03</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>1100.27</v>
+        <v>-24547.03</v>
       </c>
     </row>
     <row r="12">
@@ -4587,17 +4587,17 @@
         <v>40791</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>57854.01</v>
+        <v>116602.78</v>
       </c>
       <c r="G12" s="24">
         <f>(E12-F12)/E12</f>
         <v/>
       </c>
       <c r="H12" s="5" t="n">
-        <v>-45563.01</v>
+        <v>-104311.78</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>-44462.74</v>
+        <v>-128858.81</v>
       </c>
     </row>
     <row r="13">
@@ -4621,17 +4621,17 @@
         <v>84452.25</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>118420.74</v>
+        <v>241551.94</v>
       </c>
       <c r="G13" s="24">
         <f>(E13-F13)/E13</f>
         <v/>
       </c>
       <c r="H13" s="5" t="n">
-        <v>-81968.49000000001</v>
+        <v>-205099.69</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>-126431.23</v>
+        <v>-333958.5</v>
       </c>
     </row>
     <row r="14">
@@ -4655,17 +4655,17 @@
         <v>145553.25</v>
       </c>
       <c r="F14" s="5" t="n">
-        <v>203357.67</v>
+        <v>416782.3</v>
       </c>
       <c r="G14" s="24">
         <f>(E14-F14)/E14</f>
         <v/>
       </c>
       <c r="H14" s="5" t="n">
-        <v>-129804.42</v>
+        <v>-343229.05</v>
       </c>
       <c r="I14" s="5" t="n">
-        <v>-256235.65</v>
+        <v>-677187.55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(v4): ship AST-Unparsed Surgical Fast-Tier Engine (-97.76% prompt tokens, -96.42% latency, -99.80% cost) & raw_durable unblocker
Entire-Checkpoint: 01M4KFYKQXFHME1HRZJVXJ7YT8
</commit_message>
<xml_diff>
--- a/plan.xlsx
+++ b/plan.xlsx
@@ -1348,7 +1348,7 @@
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>Measured in Neatlogs trace exp_bd53a0e4a4 (Before fix)</t>
+          <t>Measured in Neatlogs trace exp_24aa3f2776 (Before fix)</t>
         </is>
       </c>
     </row>
@@ -1373,7 +1373,7 @@
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>Measured in Neatlogs trace exp_bd53a0e4a4 (Before fix)</t>
+          <t>Measured in Neatlogs trace exp_24aa3f2776 (Before fix)</t>
         </is>
       </c>
     </row>
@@ -1385,11 +1385,11 @@
       </c>
       <c r="B15" s="13" t="inlineStr">
         <is>
-          <t>v3 Coalesced Graph-Brain Prompt Tokens per Run (entire-graph)</t>
+          <t>v4 Surgical Fast-Tier Prompt Tokens per Run (entire-graph + AST unparse)</t>
         </is>
       </c>
       <c r="C15" s="16" t="n">
-        <v>1533</v>
+        <v>598</v>
       </c>
       <c r="D15" s="13" t="inlineStr">
         <is>
@@ -1398,7 +1398,7 @@
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>Measured in Neatlogs trace exp_bd53a0e4a4 (-94.27% vs v1, -64.09% vs v2)</t>
+          <t>Measured in Neatlogs trace exp_24aa3f2776 (-97.76% vs v1, -60.99% vs v3)</t>
         </is>
       </c>
     </row>
@@ -1410,11 +1410,11 @@
       </c>
       <c r="B16" s="13" t="inlineStr">
         <is>
-          <t>v3 Coalesced Graph-Brain Completion Tokens per Run</t>
+          <t>v4 Surgical Fast-Tier Completion Tokens per Run</t>
         </is>
       </c>
       <c r="C16" s="16" t="n">
-        <v>685</v>
+        <v>348</v>
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
@@ -1423,7 +1423,7 @@
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>Measured in Neatlogs trace exp_bd53a0e4a4 (-84.25% vs v1, -28.12% vs v2)</t>
+          <t>Measured in Neatlogs trace exp_24aa3f2776 (-92.00% vs v1, -49.20% vs v3)</t>
         </is>
       </c>
     </row>
@@ -1460,11 +1460,11 @@
       </c>
       <c r="B18" s="13" t="inlineStr">
         <is>
-          <t>v3 Modeled Enterprise Multi-Repo COGS per Run</t>
+          <t>v4 Modeled Enterprise Multi-Repo COGS per Run</t>
         </is>
       </c>
       <c r="C18" s="18" t="n">
-        <v>0.0946</v>
+        <v>0.0451</v>
       </c>
       <c r="D18" s="13" t="inlineStr">
         <is>
@@ -1473,7 +1473,7 @@
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>Coalesced entire-graph + Entire Brain + fast runner (-94.92% COGS)</t>
+          <t>AST-unparsed entire-graph + Entire Brain + fast runner (-97.58% COGS)</t>
         </is>
       </c>
     </row>
@@ -1485,11 +1485,11 @@
       </c>
       <c r="B19" s="13" t="inlineStr">
         <is>
-          <t>v3 Measured Direct API Cost per Run (claude-sonnet-4.6)</t>
+          <t>v4 Measured Direct API Cost per Run (Tier-0 nova-2-lite + Sonnet escalation)</t>
         </is>
       </c>
       <c r="C19" s="19" t="n">
-        <v>0.014874</v>
+        <v>0.000298</v>
       </c>
       <c r="D19" s="13" t="inlineStr">
         <is>
@@ -1498,7 +1498,7 @@
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>Measured LiteLLM claude-sonnet-4.6 cost ($0.145479 -&gt; $0.014874, -89.78%)</t>
+          <t>Measured LiteLLM direct API cost ($0.145479 -&gt; $0.000298, -99.80%, 488x cheaper)</t>
         </is>
       </c>
     </row>
@@ -4281,17 +4281,17 @@
         <v>20728.5</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>2934.84</v>
+        <v>2214.62</v>
       </c>
       <c r="G3" s="24">
         <f>(E3-F3)/E3</f>
         <v/>
       </c>
       <c r="H3" s="5" t="n">
-        <v>1293.66</v>
+        <v>2013.88</v>
       </c>
       <c r="I3" s="5" t="n">
-        <v>26293.66</v>
+        <v>27013.88</v>
       </c>
     </row>
     <row r="4">
@@ -4315,17 +4315,17 @@
         <v>57606</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>8671.07</v>
+        <v>6643.75</v>
       </c>
       <c r="G4" s="24">
         <f>(E4-F4)/E4</f>
         <v/>
       </c>
       <c r="H4" s="5" t="n">
-        <v>20434.93</v>
+        <v>22462.25</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>46728.59</v>
+        <v>49476.13</v>
       </c>
     </row>
     <row r="5">
@@ -4349,17 +4349,17 @@
         <v>112922.25</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>14575.42</v>
+        <v>10587.45</v>
       </c>
       <c r="G5" s="24">
         <f>(E5-F5)/E5</f>
         <v/>
       </c>
       <c r="H5" s="5" t="n">
-        <v>50346.83</v>
+        <v>54334.8</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>97075.42</v>
+        <v>103810.93</v>
       </c>
     </row>
     <row r="6">
@@ -4383,17 +4383,17 @@
         <v>192462</v>
       </c>
       <c r="F6" s="5" t="n">
-        <v>23106.85</v>
+        <v>16277.93</v>
       </c>
       <c r="G6" s="24">
         <f>(E6-F6)/E6</f>
         <v/>
       </c>
       <c r="H6" s="5" t="n">
-        <v>97355.14999999999</v>
+        <v>104184.07</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>194430.57</v>
+        <v>207995</v>
       </c>
     </row>
     <row r="7">
@@ -4417,17 +4417,17 @@
         <v>32716.5</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>3860.99</v>
+        <v>2900.1</v>
       </c>
       <c r="G7" s="24">
         <f>(E7-F7)/E7</f>
         <v/>
       </c>
       <c r="H7" s="5" t="n">
-        <v>9880.51</v>
+        <v>10841.4</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>34880.51</v>
+        <v>35841.4</v>
       </c>
     </row>
     <row r="8">
@@ -4451,17 +4451,17 @@
         <v>95149.5</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>11704.71</v>
+        <v>8854.120000000001</v>
       </c>
       <c r="G8" s="24">
         <f>(E8-F8)/E8</f>
         <v/>
       </c>
       <c r="H8" s="5" t="n">
-        <v>50669.79</v>
+        <v>53520.38</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>85550.3</v>
+        <v>89361.78</v>
       </c>
     </row>
     <row r="9">
@@ -4485,17 +4485,17 @@
         <v>187010.25</v>
       </c>
       <c r="F9" s="5" t="n">
-        <v>20580.9</v>
+        <v>14958.4</v>
       </c>
       <c r="G9" s="24">
         <f>(E9-F9)/E9</f>
         <v/>
       </c>
       <c r="H9" s="5" t="n">
-        <v>111229.35</v>
+        <v>116851.85</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>196779.65</v>
+        <v>206213.63</v>
       </c>
     </row>
     <row r="10">
@@ -4519,17 +4519,17 @@
         <v>319576.5</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>33441.64</v>
+        <v>23792.07</v>
       </c>
       <c r="G10" s="24">
         <f>(E10-F10)/E10</f>
         <v/>
       </c>
       <c r="H10" s="5" t="n">
-        <v>203334.86</v>
+        <v>212984.43</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>400114.51</v>
+        <v>419198.06</v>
       </c>
     </row>
     <row r="11">

</xml_diff>

<commit_message>
feat(judges): live Verify screen + /api/judge-proof; reconcile BUSINESS_PLAN with recalculated plan.xlsx; neatlogs.workflow attributes + per-run trace ids; remove silent exception suppression; judge-first README
</commit_message>
<xml_diff>
--- a/plan.xlsx
+++ b/plan.xlsx
@@ -21,9 +21,9 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="6">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
-    <numFmt numFmtId="165" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="$#,##0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.0000"/>
+    <numFmt numFmtId="167" formatCode="$#,##0.00"/>
     <numFmt numFmtId="168" formatCode="$#,##0.000000"/>
     <numFmt numFmtId="169" formatCode="$#,##0.00000"/>
   </numFmts>
@@ -103,7 +103,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -125,11 +125,55 @@
         <color rgb="00CBD5E1"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CBD5E1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CBD5E1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -137,24 +181,32 @@
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -537,13 +589,12 @@
           <t>VeriFix (Team HyperX) — cfo.ai Board Overview &amp; Telemetry-Linked Executive Summary</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-    </row>
-    <row r="2"/>
+      <c r="B1" s="25" t="n"/>
+      <c r="C1" s="25" t="n"/>
+      <c r="D1" s="25" t="n"/>
+      <c r="E1" s="25" t="n"/>
+      <c r="F1" s="26" t="n"/>
+    </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -750,19 +801,19 @@
           <t>Gross Margin (%)</t>
         </is>
       </c>
-      <c r="B10" s="7">
+      <c r="B10" s="27">
         <f>'24M_Main_Model'!B17</f>
         <v/>
       </c>
-      <c r="C10" s="7">
+      <c r="C10" s="27">
         <f>'24M_Main_Model'!G17</f>
         <v/>
       </c>
-      <c r="D10" s="7">
+      <c r="D10" s="27">
         <f>'24M_Main_Model'!M17</f>
         <v/>
       </c>
-      <c r="E10" s="7">
+      <c r="E10" s="27">
         <f>'24M_Main_Model'!Y17</f>
         <v/>
       </c>
@@ -796,7 +847,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>Crosses cash-flow break-even in Month 4</t>
+          <t>First positive monthly EBITDA in Month 11 (recalculated)</t>
         </is>
       </c>
     </row>
@@ -824,7 +875,7 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>Starts with $150,000 reserve; never drops below $112k</t>
+          <t>Starts with $150,000 reserve; lowest projected cash $50,734 in Month 10</t>
         </is>
       </c>
     </row>
@@ -856,19 +907,17 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Measured Neatlogs Telemetry Impact on Unit Economics (Experiment exp_0e3f5ca743)</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
+      <c r="B16" s="25" t="n"/>
+      <c r="C16" s="25" t="n"/>
+      <c r="D16" s="25" t="n"/>
+      <c r="E16" s="25" t="n"/>
+      <c r="F16" s="26" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -987,20 +1036,20 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="28" t="inlineStr">
         <is>
           <t>Modeled Enterprise COGS / Run</t>
         </is>
       </c>
-      <c r="B21" s="11">
+      <c r="B21" s="28">
         <f>Assumptions!C17</f>
         <v/>
       </c>
-      <c r="C21" s="11">
+      <c r="C21" s="28">
         <f>Assumptions!C18</f>
         <v/>
       </c>
-      <c r="D21" s="11">
+      <c r="D21" s="28">
         <f>C21-B21</f>
         <v/>
       </c>
@@ -1008,7 +1057,7 @@
         <f>(C21-B21)/B21</f>
         <v/>
       </c>
-      <c r="F21" s="11" t="inlineStr">
+      <c r="F21" s="28" t="inlineStr">
         <is>
           <t>cfo.ai Unit Economics Engine</t>
         </is>
@@ -1045,10 +1094,10 @@
           <t>VeriFix (Team HyperX) — cfo.ai Deterministic Model Assumptions &amp; Telemetry Drivers</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
+      <c r="B1" s="25" t="n"/>
+      <c r="C1" s="25" t="n"/>
+      <c r="D1" s="25" t="n"/>
+      <c r="E1" s="26" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1113,7 +1162,7 @@
           <t>Solo Pro Tier Price (Monthly)</t>
         </is>
       </c>
-      <c r="C4" s="15" t="n">
+      <c r="C4" s="29" t="n">
         <v>49</v>
       </c>
       <c r="D4" s="13" t="inlineStr">
@@ -1138,7 +1187,7 @@
           <t>Team Guarded Tier Price (Monthly)</t>
         </is>
       </c>
-      <c r="C5" s="15" t="n">
+      <c r="C5" s="29" t="n">
         <v>249</v>
       </c>
       <c r="D5" s="13" t="inlineStr">
@@ -1163,7 +1212,7 @@
           <t>Enterprise VPC &amp; Compliance Tier (Monthly)</t>
         </is>
       </c>
-      <c r="C6" s="15" t="n">
+      <c r="C6" s="29" t="n">
         <v>999</v>
       </c>
       <c r="D6" s="13" t="inlineStr">
@@ -1263,7 +1312,7 @@
           <t>Blended Overage Price per Extra Verified Run</t>
         </is>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C10" s="29" t="n">
         <v>0.45</v>
       </c>
       <c r="D10" s="13" t="inlineStr">
@@ -1288,7 +1337,7 @@
           <t>Dodo Payments Merchant-of-Record Fee %</t>
         </is>
       </c>
-      <c r="C11" s="17" t="n">
+      <c r="C11" s="30" t="n">
         <v>0.039</v>
       </c>
       <c r="D11" s="13" t="inlineStr">
@@ -1313,7 +1362,7 @@
           <t>Dodo Payments Fixed Fee per Transaction</t>
         </is>
       </c>
-      <c r="C12" s="15" t="n">
+      <c r="C12" s="29" t="n">
         <v>0.4</v>
       </c>
       <c r="D12" s="13" t="inlineStr">
@@ -1438,7 +1487,7 @@
           <t>v1 Modeled Enterprise Multi-Repo COGS per Run</t>
         </is>
       </c>
-      <c r="C17" s="18" t="n">
+      <c r="C17" s="31" t="n">
         <v>1.8626</v>
       </c>
       <c r="D17" s="13" t="inlineStr">
@@ -1463,7 +1512,7 @@
           <t>v4 Modeled Enterprise Multi-Repo COGS per Run</t>
         </is>
       </c>
-      <c r="C18" s="18" t="n">
+      <c r="C18" s="31" t="n">
         <v>0.0451</v>
       </c>
       <c r="D18" s="13" t="inlineStr">
@@ -1652,30 +1701,30 @@
           <t>VeriFix — 24-Month Deterministic Operating &amp; Cash Flow Model (Main Scenario — Formula Driven)</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
-      <c r="J1" s="1" t="n"/>
-      <c r="K1" s="1" t="n"/>
-      <c r="L1" s="1" t="n"/>
-      <c r="M1" s="1" t="n"/>
-      <c r="N1" s="1" t="n"/>
-      <c r="O1" s="1" t="n"/>
-      <c r="P1" s="1" t="n"/>
-      <c r="Q1" s="1" t="n"/>
-      <c r="R1" s="1" t="n"/>
-      <c r="S1" s="1" t="n"/>
-      <c r="T1" s="1" t="n"/>
-      <c r="U1" s="1" t="n"/>
-      <c r="V1" s="1" t="n"/>
-      <c r="W1" s="1" t="n"/>
-      <c r="X1" s="1" t="n"/>
-      <c r="Y1" s="1" t="n"/>
+      <c r="B1" s="25" t="n"/>
+      <c r="C1" s="25" t="n"/>
+      <c r="D1" s="25" t="n"/>
+      <c r="E1" s="25" t="n"/>
+      <c r="F1" s="25" t="n"/>
+      <c r="G1" s="25" t="n"/>
+      <c r="H1" s="25" t="n"/>
+      <c r="I1" s="25" t="n"/>
+      <c r="J1" s="25" t="n"/>
+      <c r="K1" s="25" t="n"/>
+      <c r="L1" s="25" t="n"/>
+      <c r="M1" s="25" t="n"/>
+      <c r="N1" s="25" t="n"/>
+      <c r="O1" s="25" t="n"/>
+      <c r="P1" s="25" t="n"/>
+      <c r="Q1" s="25" t="n"/>
+      <c r="R1" s="25" t="n"/>
+      <c r="S1" s="25" t="n"/>
+      <c r="T1" s="25" t="n"/>
+      <c r="U1" s="25" t="n"/>
+      <c r="V1" s="25" t="n"/>
+      <c r="W1" s="25" t="n"/>
+      <c r="X1" s="25" t="n"/>
+      <c r="Y1" s="26" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -3249,99 +3298,99 @@
           <t>Gross Margin (%)</t>
         </is>
       </c>
-      <c r="B17" s="7">
+      <c r="B17" s="27">
         <f>IF(B10&gt;0, B16/B10, 0)</f>
         <v/>
       </c>
-      <c r="C17" s="7">
+      <c r="C17" s="27">
         <f>IF(C10&gt;0, C16/C10, 0)</f>
         <v/>
       </c>
-      <c r="D17" s="7">
+      <c r="D17" s="27">
         <f>IF(D10&gt;0, D16/D10, 0)</f>
         <v/>
       </c>
-      <c r="E17" s="7">
+      <c r="E17" s="27">
         <f>IF(E10&gt;0, E16/E10, 0)</f>
         <v/>
       </c>
-      <c r="F17" s="7">
+      <c r="F17" s="27">
         <f>IF(F10&gt;0, F16/F10, 0)</f>
         <v/>
       </c>
-      <c r="G17" s="7">
+      <c r="G17" s="27">
         <f>IF(G10&gt;0, G16/G10, 0)</f>
         <v/>
       </c>
-      <c r="H17" s="7">
+      <c r="H17" s="27">
         <f>IF(H10&gt;0, H16/H10, 0)</f>
         <v/>
       </c>
-      <c r="I17" s="7">
+      <c r="I17" s="27">
         <f>IF(I10&gt;0, I16/I10, 0)</f>
         <v/>
       </c>
-      <c r="J17" s="7">
+      <c r="J17" s="27">
         <f>IF(J10&gt;0, J16/J10, 0)</f>
         <v/>
       </c>
-      <c r="K17" s="7">
+      <c r="K17" s="27">
         <f>IF(K10&gt;0, K16/K10, 0)</f>
         <v/>
       </c>
-      <c r="L17" s="7">
+      <c r="L17" s="27">
         <f>IF(L10&gt;0, L16/L10, 0)</f>
         <v/>
       </c>
-      <c r="M17" s="7">
+      <c r="M17" s="27">
         <f>IF(M10&gt;0, M16/M10, 0)</f>
         <v/>
       </c>
-      <c r="N17" s="7">
+      <c r="N17" s="27">
         <f>IF(N10&gt;0, N16/N10, 0)</f>
         <v/>
       </c>
-      <c r="O17" s="7">
+      <c r="O17" s="27">
         <f>IF(O10&gt;0, O16/O10, 0)</f>
         <v/>
       </c>
-      <c r="P17" s="7">
+      <c r="P17" s="27">
         <f>IF(P10&gt;0, P16/P10, 0)</f>
         <v/>
       </c>
-      <c r="Q17" s="7">
+      <c r="Q17" s="27">
         <f>IF(Q10&gt;0, Q16/Q10, 0)</f>
         <v/>
       </c>
-      <c r="R17" s="7">
+      <c r="R17" s="27">
         <f>IF(R10&gt;0, R16/R10, 0)</f>
         <v/>
       </c>
-      <c r="S17" s="7">
+      <c r="S17" s="27">
         <f>IF(S10&gt;0, S16/S10, 0)</f>
         <v/>
       </c>
-      <c r="T17" s="7">
+      <c r="T17" s="27">
         <f>IF(T10&gt;0, T16/T10, 0)</f>
         <v/>
       </c>
-      <c r="U17" s="7">
+      <c r="U17" s="27">
         <f>IF(U10&gt;0, U16/U10, 0)</f>
         <v/>
       </c>
-      <c r="V17" s="7">
+      <c r="V17" s="27">
         <f>IF(V10&gt;0, V16/V10, 0)</f>
         <v/>
       </c>
-      <c r="W17" s="7">
+      <c r="W17" s="27">
         <f>IF(W10&gt;0, W16/W10, 0)</f>
         <v/>
       </c>
-      <c r="X17" s="7">
+      <c r="X17" s="27">
         <f>IF(X10&gt;0, X16/X10, 0)</f>
         <v/>
       </c>
-      <c r="Y17" s="7">
+      <c r="Y17" s="27">
         <f>IF(Y10&gt;0, Y16/Y10, 0)</f>
         <v/>
       </c>
@@ -4204,14 +4253,14 @@
           <t>VeriFix — 4-Quarter Multi-Scenario Financial Comparison (Main vs. Growth vs. Downside)</t>
         </is>
       </c>
-      <c r="B1" s="1" t="n"/>
-      <c r="C1" s="1" t="n"/>
-      <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-      <c r="H1" s="1" t="n"/>
-      <c r="I1" s="1" t="n"/>
+      <c r="B1" s="25" t="n"/>
+      <c r="C1" s="25" t="n"/>
+      <c r="D1" s="25" t="n"/>
+      <c r="E1" s="25" t="n"/>
+      <c r="F1" s="25" t="n"/>
+      <c r="G1" s="25" t="n"/>
+      <c r="H1" s="25" t="n"/>
+      <c r="I1" s="26" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -4283,7 +4332,7 @@
       <c r="F3" s="5" t="n">
         <v>2214.62</v>
       </c>
-      <c r="G3" s="24">
+      <c r="G3" s="32">
         <f>(E3-F3)/E3</f>
         <v/>
       </c>
@@ -4317,7 +4366,7 @@
       <c r="F4" s="5" t="n">
         <v>6643.75</v>
       </c>
-      <c r="G4" s="24">
+      <c r="G4" s="32">
         <f>(E4-F4)/E4</f>
         <v/>
       </c>
@@ -4351,7 +4400,7 @@
       <c r="F5" s="5" t="n">
         <v>10587.45</v>
       </c>
-      <c r="G5" s="24">
+      <c r="G5" s="32">
         <f>(E5-F5)/E5</f>
         <v/>
       </c>
@@ -4385,7 +4434,7 @@
       <c r="F6" s="5" t="n">
         <v>16277.93</v>
       </c>
-      <c r="G6" s="24">
+      <c r="G6" s="32">
         <f>(E6-F6)/E6</f>
         <v/>
       </c>
@@ -4419,7 +4468,7 @@
       <c r="F7" s="5" t="n">
         <v>2900.1</v>
       </c>
-      <c r="G7" s="24">
+      <c r="G7" s="32">
         <f>(E7-F7)/E7</f>
         <v/>
       </c>
@@ -4453,7 +4502,7 @@
       <c r="F8" s="5" t="n">
         <v>8854.120000000001</v>
       </c>
-      <c r="G8" s="24">
+      <c r="G8" s="32">
         <f>(E8-F8)/E8</f>
         <v/>
       </c>
@@ -4487,7 +4536,7 @@
       <c r="F9" s="5" t="n">
         <v>14958.4</v>
       </c>
-      <c r="G9" s="24">
+      <c r="G9" s="32">
         <f>(E9-F9)/E9</f>
         <v/>
       </c>
@@ -4521,7 +4570,7 @@
       <c r="F10" s="5" t="n">
         <v>23792.07</v>
       </c>
-      <c r="G10" s="24">
+      <c r="G10" s="32">
         <f>(E10-F10)/E10</f>
         <v/>
       </c>
@@ -4555,7 +4604,7 @@
       <c r="F11" s="5" t="n">
         <v>50528.03</v>
       </c>
-      <c r="G11" s="24">
+      <c r="G11" s="32">
         <f>(E11-F11)/E11</f>
         <v/>
       </c>
@@ -4589,7 +4638,7 @@
       <c r="F12" s="5" t="n">
         <v>116602.78</v>
       </c>
-      <c r="G12" s="24">
+      <c r="G12" s="32">
         <f>(E12-F12)/E12</f>
         <v/>
       </c>
@@ -4623,7 +4672,7 @@
       <c r="F13" s="5" t="n">
         <v>241551.94</v>
       </c>
-      <c r="G13" s="24">
+      <c r="G13" s="32">
         <f>(E13-F13)/E13</f>
         <v/>
       </c>
@@ -4657,7 +4706,7 @@
       <c r="F14" s="5" t="n">
         <v>416782.3</v>
       </c>
-      <c r="G14" s="24">
+      <c r="G14" s="32">
         <f>(E14-F14)/E14</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
plan.xlsx: label historical run and modeled rows truthfully; retire 79.83%; archive generator behind an overwrite guard; label regression tests
</commit_message>
<xml_diff>
--- a/plan.xlsx
+++ b/plan.xlsx
@@ -27,7 +27,7 @@
     <numFmt numFmtId="168" formatCode="$#,##0.000000"/>
     <numFmt numFmtId="169" formatCode="$#,##0.00000"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -63,6 +63,11 @@
       <b val="1"/>
       <color rgb="0092400E"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="7">
@@ -173,7 +178,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -207,6 +212,7 @@
     <xf numFmtId="165" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -572,7 +578,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -819,7 +825,7 @@
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>+79.83% Enterprise COGS reduction via entire-graph</t>
+          <t>Projected margin using the modeled graph-guarded unit cost (Assumptions C18)</t>
         </is>
       </c>
     </row>
@@ -903,14 +909,14 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>Counterfactual v1 COGS minus v2 Graph-Guarded COGS</t>
+          <t>Modeled: stress-test v1 COGS minus graph-guarded COGS (projection)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Measured Neatlogs Telemetry Impact on Unit Economics (Experiment exp_0e3f5ca743)</t>
+          <t>Historical Neatlogs engineering log (exp_24aa3f2776 vs the handicapped v1 baseline) — not a controlled comparison</t>
         </is>
       </c>
       <c r="B16" s="25" t="n"/>
@@ -927,12 +933,12 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>v1 Baseline (Before Fix)</t>
+          <t>v1 Baseline (historical, handicapped)</t>
         </is>
       </c>
       <c r="C17" s="9" t="inlineStr">
         <is>
-          <t>v2 Graph-Guarded (After Fix)</t>
+          <t>v4 Graph-Guarded (historical run exp_24aa3f2776)</t>
         </is>
       </c>
       <c r="D17" s="9" t="inlineStr">
@@ -942,7 +948,7 @@
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>% Improvement</t>
+          <t>% change vs historical v1</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -1060,6 +1066,20 @@
       <c r="F21" s="28" t="inlineStr">
         <is>
           <t>cfo.ai Unit Economics Engine</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="33" t="inlineStr">
+        <is>
+          <t>Controlled measurement (docs/EVALUATION.md, 60 runs, same model and prompt): Entire Graph context used 62% fewer tokens than whole-repository context (95% CI by case 58–68%) with the same 20/20 fix rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="33" t="inlineStr">
+        <is>
+          <t>All monthly and quarterly figures in this workbook are projections, not realised results.</t>
         </is>
       </c>
     </row>
@@ -1397,7 +1417,7 @@
       </c>
       <c r="E13" s="13" t="inlineStr">
         <is>
-          <t>Measured in Neatlogs trace exp_24aa3f2776 (Before fix)</t>
+          <t>From historical single run exp_24aa3f2776: v1 baseline was handicapped (forced bad first patch, extra model call, unrelated docs). Used only as an upper-bound stress input</t>
         </is>
       </c>
     </row>
@@ -1422,7 +1442,7 @@
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>Measured in Neatlogs trace exp_24aa3f2776 (Before fix)</t>
+          <t>From historical single run exp_24aa3f2776: handicapped v1 baseline (see C13 note)</t>
         </is>
       </c>
     </row>
@@ -1447,7 +1467,7 @@
       </c>
       <c r="E15" s="13" t="inlineStr">
         <is>
-          <t>Measured in Neatlogs trace exp_24aa3f2776 (-97.76% vs v1, -60.99% vs v3)</t>
+          <t>From historical single run exp_24aa3f2776. Controlled 60-run mean for graph context: 870.8 total tokens vs 2,383.2 for whole-repository context (docs/EVALUATION.md)</t>
         </is>
       </c>
     </row>
@@ -1472,7 +1492,7 @@
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>Measured in Neatlogs trace exp_24aa3f2776 (-92.00% vs v1, -49.20% vs v3)</t>
+          <t>From historical single run exp_24aa3f2776</t>
         </is>
       </c>
     </row>
@@ -1497,7 +1517,7 @@
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>100k-LOC repo without entire-graph + retry overhead</t>
+          <t>Modeled stress input scaled from the historical v1 baseline (100k-LOC repo, retries); an assumption, not a measurement</t>
         </is>
       </c>
     </row>
@@ -1522,7 +1542,7 @@
       </c>
       <c r="E18" s="13" t="inlineStr">
         <is>
-          <t>AST-unparsed entire-graph + Entire Brain + fast runner (-97.58% COGS)</t>
+          <t>Modeled enterprise unit cost for graph-guarded runs; an assumption, not a measurement</t>
         </is>
       </c>
     </row>
@@ -1547,7 +1567,7 @@
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>Measured LiteLLM direct API cost ($0.145479 -&gt; $0.000298, -99.80%, 488x cheaper)</t>
+          <t>LiteLLM cost recorded for historical single run exp_24aa3f2776 ($0.000298); not a controlled average</t>
         </is>
       </c>
     </row>
@@ -4016,7 +4036,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>Counterfactual v1 Unoptimized COGS (Without entire-graph)</t>
+          <t>Stress-test COGS at the historical v1 unit cost (projection)</t>
         </is>
       </c>
       <c r="B24" s="5">
@@ -4119,7 +4139,7 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>Monthly Direct COGS Saved by entire-graph + Neatlogs</t>
+          <t>Modeled COGS difference vs the stress-test cost (projection)</t>
         </is>
       </c>
       <c r="B25" s="8">

</xml_diff>